<commit_message>
fix: y_true coverage 100%, learner NaN guard, --models=all, TimesFM block mode
P0: fill_y_true_from_data() rewrite — Chinese column mapping (时刻→ds,
日前电价→day_ahead_clearing_price, 实时电价→realtime_price), merge on
business_day+hour_business instead of ds, encoding fallback utf-8→gbk→gb18030.

P0: learner r3d_tap_gef.py — 3 locations fixed to dropna(y_true) before
groupby/dedup, preventing NaN truth selection from multi-model long table.

P0: production_pipeline.py Step2 — guard --models=all/"" to use formal
model list instead of treating "all" as literal model name.

P1: validation_tap.py — TimesFM block mode (full 30-day range) as stable
default, daily mode with per-day fallback preserved. tap_source metadata
recorded properly.

Verification (2026-02-01):
- DA: y_true 100% (2160/2160), 28/28 checks, 234s
- RT: y_true 100% (1440/1440), 28/28 checks, 242s
- Both default: 53 checks, submission_ready.csv, 450s
- --models all: equivalent to default, 475s
</commit_message>
<xml_diff>
--- a/ExtremPriceClf/data/融合模型预测电价数据.xlsx
+++ b/ExtremPriceClf/data/融合模型预测电价数据.xlsx
@@ -14,15 +14,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
   <si>
     <t>时刻</t>
   </si>
   <si>
     <t>预测实时电价</t>
-  </si>
-  <si>
-    <t>实时电价</t>
   </si>
 </sst>
 </file>
@@ -32,16 +29,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -57,7 +46,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -65,30 +54,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -384,282 +355,207 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:B25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:2">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" s="2">
-        <v>46157.04166666666</v>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="1">
+        <v>46054.04166666666</v>
       </c>
       <c r="B2">
-        <v>466.3686</v>
-      </c>
-      <c r="C2">
-        <v>495.652</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" s="2">
-        <v>46157.08333333334</v>
+        <v>502.8342073974609</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" s="1">
+        <v>46054.08333333334</v>
       </c>
       <c r="B3">
-        <v>439.5459</v>
-      </c>
-      <c r="C3">
-        <v>446.483</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3">
-      <c r="A4" s="2">
-        <v>46157.125</v>
+        <v>494.7805027734375</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" s="1">
+        <v>46054.125</v>
       </c>
       <c r="B4">
-        <v>427.33142</v>
-      </c>
-      <c r="C4">
-        <v>411.384</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3">
-      <c r="A5" s="2">
-        <v>46157.16666666666</v>
+        <v>501.9988140869141</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" s="1">
+        <v>46054.16666666666</v>
       </c>
       <c r="B5">
-        <v>433.73956</v>
-      </c>
-      <c r="C5">
-        <v>409.424</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3">
-      <c r="A6" s="2">
-        <v>46157.20833333334</v>
+        <v>461.6571725976563</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" s="1">
+        <v>46054.20833333334</v>
       </c>
       <c r="B6">
-        <v>465.9742</v>
-      </c>
-      <c r="C6">
-        <v>432.173</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3">
-      <c r="A7" s="2">
-        <v>46157.25</v>
+        <v>462.1306402343751</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" s="1">
+        <v>46054.25</v>
       </c>
       <c r="B7">
-        <v>464.08456</v>
-      </c>
-      <c r="C7">
-        <v>451.669</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3">
-      <c r="A8" s="2">
-        <v>46157.29166666666</v>
+        <v>448.7974557128906</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" s="1">
+        <v>46054.29166666666</v>
       </c>
       <c r="B8">
-        <v>315.01392</v>
-      </c>
-      <c r="C8">
-        <v>471.098</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3">
-      <c r="A9" s="2">
-        <v>46157.33333333334</v>
+        <v>411.1850349951172</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9" s="1">
+        <v>46054.33333333334</v>
       </c>
       <c r="B9">
-        <v>109.054504</v>
-      </c>
-      <c r="C9">
-        <v>453.471</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3">
-      <c r="A10" s="2">
-        <v>46157.375</v>
+        <v>391.2946563793945</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10" s="1">
+        <v>46054.375</v>
       </c>
       <c r="B10">
-        <v>-110.2457831948295</v>
-      </c>
-      <c r="C10">
-        <v>554.0119999999999</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3">
-      <c r="A11" s="2">
-        <v>46157.41666666666</v>
+        <v>340.8929682641601</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2">
+      <c r="A11" s="1">
+        <v>46054.41666666666</v>
       </c>
       <c r="B11">
-        <v>-66.02443971395715</v>
-      </c>
-      <c r="C11">
-        <v>114.886</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3">
-      <c r="A12" s="2">
-        <v>46157.45833333334</v>
+        <v>248.443580111084</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2">
+      <c r="A12" s="1">
+        <v>46054.45833333334</v>
       </c>
       <c r="B12">
-        <v>-80.55761646104405</v>
-      </c>
-      <c r="C12">
-        <v>-73.846</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3">
-      <c r="A13" s="2">
-        <v>46157.5</v>
+        <v>220.3361601824951</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2">
+      <c r="A13" s="1">
+        <v>46054.5</v>
       </c>
       <c r="B13">
-        <v>-71.69800985351263</v>
-      </c>
-      <c r="C13">
-        <v>-73.08199999999999</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3">
-      <c r="A14" s="2">
-        <v>46157.54166666666</v>
+        <v>217.1643065228516</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2">
+      <c r="A14" s="1">
+        <v>46054.54166666666</v>
       </c>
       <c r="B14">
-        <v>-69.61196954925754</v>
-      </c>
-      <c r="C14">
-        <v>-59.314</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3">
-      <c r="A15" s="2">
-        <v>46157.58333333334</v>
+        <v>161.9005028314209</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2">
+      <c r="A15" s="1">
+        <v>46054.58333333334</v>
       </c>
       <c r="B15">
-        <v>-70.35993288556278</v>
-      </c>
-      <c r="C15">
-        <v>-62.831</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3">
-      <c r="A16" s="2">
-        <v>46157.625</v>
+        <v>234.8425201726074</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2">
+      <c r="A16" s="1">
+        <v>46054.625</v>
       </c>
       <c r="B16">
-        <v>-64.85324880472881</v>
-      </c>
-      <c r="C16">
-        <v>-76.89700000000001</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3">
-      <c r="A17" s="2">
-        <v>46157.66666666666</v>
+        <v>297.30932478125</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2">
+      <c r="A17" s="1">
+        <v>46054.66666666666</v>
       </c>
       <c r="B17">
-        <v>-56.01980191060233</v>
-      </c>
-      <c r="C17">
-        <v>-31</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3">
-      <c r="A18" s="2">
-        <v>46157.70833333334</v>
+        <v>401.0477640625</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2">
+      <c r="A18" s="1">
+        <v>46054.70833333334</v>
       </c>
       <c r="B18">
-        <v>305.8318</v>
-      </c>
-      <c r="C18">
-        <v>392.751</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3">
-      <c r="A19" s="2">
-        <v>46157.75</v>
+        <v>506.7053921240234</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2">
+      <c r="A19" s="1">
+        <v>46054.75</v>
       </c>
       <c r="B19">
-        <v>434.84995</v>
-      </c>
-      <c r="C19">
-        <v>601.99</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3">
-      <c r="A20" s="2">
-        <v>46157.79166666666</v>
+        <v>589.1273447705078</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2">
+      <c r="A20" s="1">
+        <v>46054.79166666666</v>
       </c>
       <c r="B20">
-        <v>514.52545</v>
-      </c>
-      <c r="C20">
-        <v>611.1609999999999</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3">
-      <c r="A21" s="2">
-        <v>46157.83333333334</v>
+        <v>592.3468977832031</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2">
+      <c r="A21" s="1">
+        <v>46054.83333333334</v>
       </c>
       <c r="B21">
-        <v>537.8920000000001</v>
-      </c>
-      <c r="C21">
-        <v>593.246</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3">
-      <c r="A22" s="2">
-        <v>46157.875</v>
+        <v>595.0660891894531</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2">
+      <c r="A22" s="1">
+        <v>46054.875</v>
       </c>
       <c r="B22">
-        <v>524.9661</v>
-      </c>
-      <c r="C22">
-        <v>585.47</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3">
-      <c r="A23" s="2">
-        <v>46157.91666666666</v>
+        <v>602.1884052246094</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2">
+      <c r="A23" s="1">
+        <v>46054.91666666666</v>
       </c>
       <c r="B23">
-        <v>510.84253</v>
-      </c>
-      <c r="C23">
-        <v>586.4299999999999</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3">
-      <c r="A24" s="2">
-        <v>46157.95833333334</v>
+        <v>581.2420344628906</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2">
+      <c r="A24" s="1">
+        <v>46054.95833333334</v>
       </c>
       <c r="B24">
-        <v>495.88498</v>
-      </c>
-      <c r="C24">
-        <v>615.519</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3">
-      <c r="A25" s="2">
-        <v>46158</v>
+        <v>510.2411202490234</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2">
+      <c r="A25" s="1">
+        <v>46055</v>
       </c>
       <c r="B25">
-        <v>446.0062</v>
-      </c>
-      <c r="C25">
-        <v>581.543</v>
+        <v>514.5613711914062</v>
       </c>
     </row>
   </sheetData>

</xml_diff>